<commit_message>
fix: validate EANs as EAN-13 instead of ignoring leading zeros in Bexio
An EAN is always an EAN-13, so the parser now checks every EAN with
Nager.ArticleNumber. Shorter codes first get the leading zeros back that
Excel drops from number cells (826710896036 becomes 0826710896036); an EAN
that is still no valid EAN-13 stops reading the file with its row.

The Bexio lookup compares the intern_code exactly again:
LeadingZeroEanArticleMatcher, FallbackArticleMatcher and
ArticleMatch.IsMissing are removed. The fixture EAN 7612345678904 had a
wrong check digit and is now 7612345678900; row 9 holds 826710896036 as a
number cell.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/BexioOrderImport.Format.EanList.Tests/Fixtures/EanListOrder.xlsx
+++ b/src/BexioOrderImport.Format.EanList.Tests/Fixtures/EanListOrder.xlsx
@@ -401,7 +401,7 @@
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0">
-        <x:v>7612345678904</x:v>
+        <x:v>7612345678900</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>3</x:v>
@@ -449,7 +449,7 @@
     </x:row>
     <x:row r="9" spans="1:4">
       <x:c r="A9" s="0">
-        <x:v>7612345678904</x:v>
+        <x:v>826710896036</x:v>
       </x:c>
       <x:c r="B9" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
fix: validate EANs as EAN-13 and restore missing leading zeros (#26)
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/BexioOrderImport.Format.EanList.Tests/Fixtures/EanListOrder.xlsx
+++ b/src/BexioOrderImport.Format.EanList.Tests/Fixtures/EanListOrder.xlsx
@@ -401,7 +401,7 @@
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0">
-        <x:v>7612345678904</x:v>
+        <x:v>7612345678900</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>3</x:v>
@@ -449,7 +449,7 @@
     </x:row>
     <x:row r="9" spans="1:4">
       <x:c r="A9" s="0">
-        <x:v>7612345678904</x:v>
+        <x:v>826710896036</x:v>
       </x:c>
       <x:c r="B9" s="0">
         <x:v>5</x:v>

</xml_diff>